<commit_message>
Update YAYOBE Auto Insurance  Information .xlsx
</commit_message>
<xml_diff>
--- a/YAYOBE Auto Insurance  Information .xlsx
+++ b/YAYOBE Auto Insurance  Information .xlsx
@@ -39953,8 +39953,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B579D029B9EEEF43BF7134B87E910FFD" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="04a8eba1b9eb67d123991dece900ff02">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="84e3566b-9959-4639-85ba-5bd0fed52c65" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="baa803815429a2606699dccee3eb5277" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B579D029B9EEEF43BF7134B87E910FFD" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="41d6b042a7726b7f859b481544114349">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="84e3566b-9959-4639-85ba-5bd0fed52c65" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f11b327ec275444282ad34423527f0b" ns2:_="">
     <xsd:import namespace="84e3566b-9959-4639-85ba-5bd0fed52c65"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -40150,21 +40150,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C39D993B-CA62-47B5-8EB7-BADDD6A4CAE7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="84e3566b-9959-4639-85ba-5bd0fed52c65"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37A75B37-4E8A-47CF-8F63-B29E140BC0D6}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>